<commit_message>
added new study structure document, shared by email
</commit_message>
<xml_diff>
--- a/documents/TimeTracking_Home_MasterThesis.xlsx
+++ b/documents/TimeTracking_Home_MasterThesis.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BFH\MSE\MasterThesis\documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BFH\MSE\MSE_MasterThesis\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B484D3B0-1121-4FF6-91CD-49639C740AE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6712706E-12E4-4CDE-B76C-20CB5E861FC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="12">
   <si>
     <t>Date</t>
   </si>
@@ -60,6 +61,18 @@
   </si>
   <si>
     <t>first Meeting preparation and Meeting</t>
+  </si>
+  <si>
+    <t>Work on first document, refine phases and milestones</t>
+  </si>
+  <si>
+    <t>Start</t>
+  </si>
+  <si>
+    <t>End</t>
+  </si>
+  <si>
+    <t>Weniger ca 45 Min</t>
   </si>
 </sst>
 </file>
@@ -95,9 +108,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -378,7 +392,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7890625" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
@@ -386,7 +400,7 @@
     <col min="4" max="4" width="85.7890625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -399,8 +413,14 @@
       <c r="D1" t="s">
         <v>2</v>
       </c>
+      <c r="E1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F1" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="1">
         <v>46283</v>
       </c>
@@ -414,7 +434,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="1">
         <v>46291</v>
       </c>
@@ -428,7 +448,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="1">
         <v>46292</v>
       </c>
@@ -436,10 +456,33 @@
         <v>4</v>
       </c>
       <c r="C4">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D4" t="s">
         <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A5" s="1">
+        <v>46298</v>
+      </c>
+      <c r="B5" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5">
+        <v>3.25</v>
+      </c>
+      <c r="D5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="2">
+        <v>0.3888888888888889</v>
+      </c>
+      <c r="F5" s="2">
+        <v>0.54861111111111116</v>
+      </c>
+      <c r="G5" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added titlepages and updated gitignore
</commit_message>
<xml_diff>
--- a/documents/TimeTracking_Home_MasterThesis.xlsx
+++ b/documents/TimeTracking_Home_MasterThesis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BFH\MSE\MSE_MasterThesis\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6712706E-12E4-4CDE-B76C-20CB5E861FC1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB88FDC8-BF49-4E0F-AA25-F5173C6CD8EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="13">
   <si>
     <t>Date</t>
   </si>
@@ -73,6 +73,9 @@
   </si>
   <si>
     <t>Weniger ca 45 Min</t>
+  </si>
+  <si>
+    <t>Work on initial Thesis Document version, create the new document and remove outdated content of P1 and P2</t>
   </si>
 </sst>
 </file>
@@ -392,7 +395,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7890625" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
@@ -485,6 +488,20 @@
         <v>11</v>
       </c>
     </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A6" s="1">
+        <v>46298</v>
+      </c>
+      <c r="B6" t="s">
+        <v>4</v>
+      </c>
+      <c r="D6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="2">
+        <v>0.57638888888888884</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
reviewed only the files of chapters 1 to 2, chapter 3 not touched, also those will need reviewing not only creating files
</commit_message>
<xml_diff>
--- a/documents/TimeTracking_Home_MasterThesis.xlsx
+++ b/documents/TimeTracking_Home_MasterThesis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BFH\MSE\MSE_MasterThesis\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB88FDC8-BF49-4E0F-AA25-F5173C6CD8EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{606D672A-7C7D-45E2-A6C0-8370CF03884F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="14">
   <si>
     <t>Date</t>
   </si>
@@ -76,6 +76,9 @@
   </si>
   <si>
     <t>Work on initial Thesis Document version, create the new document and remove outdated content of P1 and P2</t>
+  </si>
+  <si>
+    <t>Restructure Document, remove chapters which are not part of Master Thesis</t>
   </si>
 </sst>
 </file>
@@ -395,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7890625" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
@@ -495,11 +498,37 @@
       <c r="B6" t="s">
         <v>4</v>
       </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
       <c r="D6" t="s">
         <v>12</v>
       </c>
       <c r="E6" s="2">
         <v>0.57638888888888884</v>
+      </c>
+      <c r="F6" s="2">
+        <v>0.61805555555555558</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A7" s="1">
+        <v>46298</v>
+      </c>
+      <c r="B7" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7" s="2">
+        <v>0.88541666666666663</v>
+      </c>
+      <c r="F7" s="2">
+        <v>0.92708333333333337</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add todo tags and some chapter checklist
</commit_message>
<xml_diff>
--- a/documents/TimeTracking_Home_MasterThesis.xlsx
+++ b/documents/TimeTracking_Home_MasterThesis.xlsx
@@ -8,15 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BFH\MSE\MSE_MasterThesis\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{606D672A-7C7D-45E2-A6C0-8370CF03884F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D30803EA-D378-487C-BE50-35EC4CBBDBB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2196" yWindow="2196" windowWidth="17280" windowHeight="10038" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="15">
   <si>
     <t>Date</t>
   </si>
@@ -79,6 +78,9 @@
   </si>
   <si>
     <t>Restructure Document, remove chapters which are not part of Master Thesis</t>
+  </si>
+  <si>
+    <t>Restructure Document, add Chapters and add Todo Tags</t>
   </si>
 </sst>
 </file>
@@ -398,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7890625" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
@@ -531,6 +533,20 @@
         <v>0.92708333333333337</v>
       </c>
     </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A8" s="1">
+        <v>46299</v>
+      </c>
+      <c r="B8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" s="2">
+        <v>0.375</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
signed document and updated timetracking
</commit_message>
<xml_diff>
--- a/documents/TimeTracking_Home_MasterThesis.xlsx
+++ b/documents/TimeTracking_Home_MasterThesis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BFH\MSE\MSE_MasterThesis\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D30803EA-D378-487C-BE50-35EC4CBBDBB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4B75BD3-80A3-45BB-A7AD-C87113853BF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2196" yWindow="2196" windowWidth="17280" windowHeight="10038" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -80,7 +80,7 @@
     <t>Restructure Document, remove chapters which are not part of Master Thesis</t>
   </si>
   <si>
-    <t>Restructure Document, add Chapters and add Todo Tags</t>
+    <t>Restructure Document, add Chapters and add Todo Tags , Sweeping Miroboard, Tasks for Monday</t>
   </si>
 </sst>
 </file>
@@ -540,11 +540,17 @@
       <c r="B8" t="s">
         <v>4</v>
       </c>
+      <c r="C8">
+        <v>2</v>
+      </c>
       <c r="D8" t="s">
         <v>14</v>
       </c>
       <c r="E8" s="2">
         <v>0.375</v>
+      </c>
+      <c r="F8" s="2">
+        <v>0.46527777777777779</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
rework on initial thesis description
</commit_message>
<xml_diff>
--- a/documents/TimeTracking_Home_MasterThesis.xlsx
+++ b/documents/TimeTracking_Home_MasterThesis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BFH\MSE\MSE_MasterThesis\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4B75BD3-80A3-45BB-A7AD-C87113853BF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8793D432-55F8-4AB0-80C0-41D26E82F128}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2196" yWindow="2196" windowWidth="17280" windowHeight="10038" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="16">
   <si>
     <t>Date</t>
   </si>
@@ -81,6 +81,9 @@
   </si>
   <si>
     <t>Restructure Document, add Chapters and add Todo Tags , Sweeping Miroboard, Tasks for Monday</t>
+  </si>
+  <si>
+    <t>Work on Introduction, rework when to state that it is 3 projects , Rework the descriptive Document</t>
   </si>
 </sst>
 </file>
@@ -400,7 +403,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7890625" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
@@ -553,6 +556,20 @@
         <v>0.46527777777777779</v>
       </c>
     </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A9" s="1">
+        <v>46305</v>
+      </c>
+      <c r="B9" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9">
+        <v>2</v>
+      </c>
+      <c r="D9" t="s">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
adding new documents for thesis to project relation
</commit_message>
<xml_diff>
--- a/documents/TimeTracking_Home_MasterThesis.xlsx
+++ b/documents/TimeTracking_Home_MasterThesis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BFH\MSE\MSE_MasterThesis\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8793D432-55F8-4AB0-80C0-41D26E82F128}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EC22931-CE46-4F68-982F-CCEBC5E48E28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2196" yWindow="2196" windowWidth="17280" windowHeight="10038" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="17">
   <si>
     <t>Date</t>
   </si>
@@ -84,6 +84,9 @@
   </si>
   <si>
     <t>Work on Introduction, rework when to state that it is 3 projects , Rework the descriptive Document</t>
+  </si>
+  <si>
+    <t>Work on Introduction, write part for 3 staged work</t>
   </si>
 </sst>
 </file>
@@ -403,7 +406,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7890625" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
@@ -570,6 +573,17 @@
         <v>15</v>
       </c>
     </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A10" s="1">
+        <v>46306</v>
+      </c>
+      <c r="B10" t="s">
+        <v>4</v>
+      </c>
+      <c r="D10" t="s">
+        <v>16</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
reviewed up to the project management methods section, but stuck there
</commit_message>
<xml_diff>
--- a/documents/TimeTracking_Home_MasterThesis.xlsx
+++ b/documents/TimeTracking_Home_MasterThesis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BFH\MSE\MSE_MasterThesis\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EC22931-CE46-4F68-982F-CCEBC5E48E28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{998BD68E-1A2F-4520-9920-A63EC865F5FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2196" yWindow="2196" windowWidth="17280" windowHeight="10038" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,6 +16,7 @@
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="18">
   <si>
     <t>Date</t>
   </si>
@@ -87,6 +88,9 @@
   </si>
   <si>
     <t>Work on Introduction, write part for 3 staged work</t>
+  </si>
+  <si>
+    <t>Work on Introduction, then continue on Project management, adding the updates since project 2</t>
   </si>
 </sst>
 </file>
@@ -406,7 +410,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7890625" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
@@ -580,8 +584,25 @@
       <c r="B10" t="s">
         <v>4</v>
       </c>
+      <c r="C10">
+        <v>2</v>
+      </c>
       <c r="D10" t="s">
         <v>16</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A11" s="1">
+        <v>46312</v>
+      </c>
+      <c r="B11" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11">
+        <v>5</v>
+      </c>
+      <c r="D11" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updates along timetracking and efforts, rewritten structure, missing corrections and adding the table as required
</commit_message>
<xml_diff>
--- a/documents/TimeTracking_Home_MasterThesis.xlsx
+++ b/documents/TimeTracking_Home_MasterThesis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BFH\MSE\MSE_MasterThesis\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{998BD68E-1A2F-4520-9920-A63EC865F5FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBB87FEF-7B2A-4AD3-B7CC-0A2B449E6F85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2196" yWindow="2196" windowWidth="17280" windowHeight="10038" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="22">
   <si>
     <t>Date</t>
   </si>
@@ -91,6 +91,18 @@
   </si>
   <si>
     <t>Work on Introduction, then continue on Project management, adding the updates since project 2</t>
+  </si>
+  <si>
+    <t>Write on Effort Planning and Review</t>
+  </si>
+  <si>
+    <t>Review what the content of Effort Planning and Review should be</t>
+  </si>
+  <si>
+    <t>Project Management</t>
+  </si>
+  <si>
+    <t>Miro Setup regarding dates, setup of Milestones timelines in excel to get phases efforts</t>
   </si>
 </sst>
 </file>
@@ -410,7 +422,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7890625" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
@@ -605,6 +617,81 @@
         <v>17</v>
       </c>
     </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A12" s="1">
+        <v>46313</v>
+      </c>
+      <c r="B12" t="s">
+        <v>4</v>
+      </c>
+      <c r="D12" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A13" s="1">
+        <v>46313</v>
+      </c>
+      <c r="B13" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A14" s="1">
+        <v>46317</v>
+      </c>
+      <c r="B14" t="s">
+        <v>4</v>
+      </c>
+      <c r="C14">
+        <v>0.5</v>
+      </c>
+      <c r="D14" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A15" s="1">
+        <v>46317</v>
+      </c>
+      <c r="B15" t="s">
+        <v>4</v>
+      </c>
+      <c r="C15">
+        <v>0.25</v>
+      </c>
+      <c r="D15" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.55000000000000004">
+      <c r="A16" s="1">
+        <v>46318</v>
+      </c>
+      <c r="B16" t="s">
+        <v>4</v>
+      </c>
+      <c r="C16">
+        <v>0.5</v>
+      </c>
+      <c r="D16" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A17" s="1">
+        <v>46318</v>
+      </c>
+      <c r="B17" t="s">
+        <v>4</v>
+      </c>
+      <c r="C17">
+        <v>1.5</v>
+      </c>
+      <c r="D17" t="s">
+        <v>21</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
time effort planning and review written in V1
</commit_message>
<xml_diff>
--- a/documents/TimeTracking_Home_MasterThesis.xlsx
+++ b/documents/TimeTracking_Home_MasterThesis.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BFH\MSE\MSE_MasterThesis\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBB87FEF-7B2A-4AD3-B7CC-0A2B449E6F85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2AE24DC-F443-4F2B-A205-7E95D6A926F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2196" yWindow="2196" windowWidth="17280" windowHeight="10038" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2532" yWindow="2532" windowWidth="17280" windowHeight="10038" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="25">
   <si>
     <t>Date</t>
   </si>
@@ -103,6 +103,15 @@
   </si>
   <si>
     <t>Miro Setup regarding dates, setup of Milestones timelines in excel to get phases efforts</t>
+  </si>
+  <si>
+    <t>Start the Phases calculation,</t>
+  </si>
+  <si>
+    <t>Write the Use case</t>
+  </si>
+  <si>
+    <t>Continue on Phases calculation, includes relative %, but also number of hours per week and expected effort, however expected hours are not used</t>
   </si>
 </sst>
 </file>
@@ -422,7 +431,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7890625" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
@@ -624,6 +633,9 @@
       <c r="B12" t="s">
         <v>4</v>
       </c>
+      <c r="C12">
+        <v>3</v>
+      </c>
       <c r="D12" t="s">
         <v>20</v>
       </c>
@@ -635,6 +647,12 @@
       <c r="B13" t="s">
         <v>4</v>
       </c>
+      <c r="C13">
+        <v>2.5</v>
+      </c>
+      <c r="D13" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" s="1">
@@ -678,7 +696,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.55000000000000004">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" s="1">
         <v>46318</v>
       </c>
@@ -690,6 +708,34 @@
       </c>
       <c r="D17" t="s">
         <v>21</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A18" s="1">
+        <v>46319</v>
+      </c>
+      <c r="B18" t="s">
+        <v>4</v>
+      </c>
+      <c r="C18">
+        <v>2</v>
+      </c>
+      <c r="D18" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A19" s="1">
+        <v>46319</v>
+      </c>
+      <c r="B19" t="s">
+        <v>4</v>
+      </c>
+      <c r="D19" t="s">
+        <v>24</v>
+      </c>
+      <c r="E19" s="2">
+        <v>0.49652777777777779</v>
       </c>
     </row>
   </sheetData>

</xml_diff>